<commit_message>
Add comprehensive tests for certification search and routing validation
- Implemented `test_buscar_certificaciones.py` to verify the search functionality for certification files.
- Created `test_ejecutables_enrutamiento.py` to validate routing for executable services, ensuring they point to the correct directories.
- Developed `test_enrutamiento_completo.py` to perform a complete dynamic routing test across all project modules, confirming proper configuration for dynamic paths.
</commit_message>
<xml_diff>
--- a/Assets/Formatos/Formato Oficial.xlsx
+++ b/Assets/Formatos/Formato Oficial.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11460"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="HU83627" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
   <si>
     <t>1.  INFORMACIÓN GENERAL DEL DESARROLLO</t>
   </si>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>Observaciones:</t>
+  </si>
+  <si>
+    <t>Todos los casos de prueba se encuentran en estado Closed por obsolescencia, tras realizar la validación correspondiente y el reporte de los hallazgos identificados.</t>
   </si>
   <si>
     <t>NOTA:  Se informa a los usuarios que después de la fecha final de la última ejecución; si no es remitido el formato con las respectivas observaciones, se dará por entendido que no presenta novedades, y se procederá a cerrar el proyecto bajo la responsabilidad del usuario.</t>
@@ -137,7 +140,7 @@
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="[$-409]dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,13 +192,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -838,129 +834,129 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1062,16 +1058,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="22" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1116,7 +1112,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1652,7 +1648,9 @@
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="24"/>
-      <c r="F15" s="25"/>
+      <c r="F15" s="25" t="s">
+        <v>10</v>
+      </c>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
       <c r="I15" s="19"/>
@@ -1663,7 +1661,7 @@
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="26" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D16" s="27"/>
       <c r="E16" s="27"/>
@@ -1691,7 +1689,7 @@
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="28" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D18" s="29"/>
       <c r="E18" s="29"/>
@@ -1719,19 +1717,19 @@
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="30" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H20" s="10"/>
       <c r="I20" s="11"/>
@@ -1744,7 +1742,7 @@
       <c r="C21" s="33"/>
       <c r="D21" s="34"/>
       <c r="E21" s="34" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F21" s="34"/>
       <c r="G21" s="35">
@@ -1759,16 +1757,16 @@
       <c r="A22" s="32"/>
       <c r="B22" s="32"/>
       <c r="C22" s="37" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D22" s="29"/>
       <c r="E22" s="29"/>
       <c r="F22" s="29"/>
       <c r="G22" s="38" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H22" s="39" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I22" s="11"/>
       <c r="J22" s="32"/>
@@ -1780,7 +1778,7 @@
       <c r="E23" s="29"/>
       <c r="F23" s="29"/>
       <c r="G23" s="38" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H23" s="39"/>
       <c r="I23" s="11"/>
@@ -1789,7 +1787,7 @@
       <c r="A24" s="40"/>
       <c r="B24" s="40"/>
       <c r="C24" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
@@ -1817,19 +1815,19 @@
       <c r="A26" s="32"/>
       <c r="B26" s="32"/>
       <c r="C26" s="30" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D26" s="31" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H26" s="10"/>
       <c r="I26" s="11"/>
@@ -1853,13 +1851,13 @@
       <c r="A28" s="42"/>
       <c r="B28" s="42"/>
       <c r="C28" s="43" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D28" s="44"/>
       <c r="E28" s="44"/>
       <c r="F28" s="44"/>
       <c r="G28" s="45" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H28" s="46"/>
       <c r="I28" s="11"/>
@@ -1874,7 +1872,7 @@
       <c r="E29" s="44"/>
       <c r="F29" s="44"/>
       <c r="G29" s="45" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H29" s="46"/>
       <c r="I29" s="11"/>

</xml_diff>